<commit_message>
fix: sheets header name
</commit_message>
<xml_diff>
--- a/public/files/IQMY-Alpro eResult Checking List 11Sept2025.xlsx
+++ b/public/files/IQMY-Alpro eResult Checking List 11Sept2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\blood-stream-v1\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FFB0BDA-32F1-4AAC-B1D0-35DAF5366038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D7760E-36C4-4C89-B67D-FD466DC50179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3CA47CF7-F541-4479-BE1B-2E5AF2DF364A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3CA47CF7-F541-4479-BE1B-2E5AF2DF364A}"/>
   </bookViews>
   <sheets>
     <sheet name="9-11 Sept" sheetId="2" r:id="rId1"/>
@@ -36,25 +36,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="2">
   <si>
     <t>Lab Number</t>
   </si>
   <si>
     <t>Prefix</t>
   </si>
-  <si>
-    <t>PREFIX</t>
-  </si>
-  <si>
-    <t>NUM</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -71,14 +65,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -104,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -113,7 +99,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1772,11 +1757,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>3</v>
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>